<commit_message>
minor updates to BLS queries and ACS data pulls
</commit_message>
<xml_diff>
--- a/Indicator_Gen/Python Code/BLS/config/BLS Configuration File.xlsx
+++ b/Indicator_Gen/Python Code/BLS/config/BLS Configuration File.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\Python Code\BLS\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C2E0F0-9043-49B4-BF04-7B68E9C0F4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF2F604-F4B4-4818-B0F9-5D7F69794DBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="2400" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="5" r:id="rId1"/>
@@ -3515,7 +3515,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor theme="4"/>
   </sheetPr>
   <dimension ref="A1:G344"/>
@@ -3587,7 +3587,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>91</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>93</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -3646,7 +3646,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -3657,7 +3657,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>102</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>104</v>
       </c>
@@ -3679,7 +3679,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>106</v>
       </c>
@@ -3690,7 +3690,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>108</v>
       </c>
@@ -3701,7 +3701,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>110</v>
       </c>
@@ -3712,7 +3712,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>112</v>
       </c>
@@ -3723,7 +3723,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>114</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>116</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>118</v>
       </c>
@@ -3773,7 +3773,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>123</v>
       </c>
@@ -3784,7 +3784,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>125</v>
       </c>
@@ -3795,7 +3795,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>127</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>129</v>
       </c>
@@ -3817,7 +3817,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>131</v>
       </c>
@@ -3828,7 +3828,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>133</v>
       </c>
@@ -3839,7 +3839,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>135</v>
       </c>
@@ -3850,7 +3850,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>137</v>
       </c>
@@ -3861,7 +3861,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>139</v>
       </c>
@@ -3872,7 +3872,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>141</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>143</v>
       </c>
@@ -3894,7 +3894,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>145</v>
       </c>
@@ -3905,7 +3905,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>147</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>151</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>153</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>155</v>
       </c>
@@ -3966,7 +3966,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>157</v>
       </c>
@@ -3977,7 +3977,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>159</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>161</v>
       </c>
@@ -3999,7 +3999,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>163</v>
       </c>
@@ -4010,7 +4010,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>165</v>
       </c>
@@ -4021,7 +4021,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>167</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>169</v>
       </c>
@@ -4043,7 +4043,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>171</v>
       </c>
@@ -4054,7 +4054,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>173</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>175</v>
       </c>
@@ -4076,7 +4076,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>177</v>
       </c>
@@ -4087,7 +4087,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>179</v>
       </c>
@@ -4098,7 +4098,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>181</v>
       </c>
@@ -4109,7 +4109,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>183</v>
       </c>
@@ -4120,7 +4120,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>185</v>
       </c>
@@ -4131,7 +4131,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>187</v>
       </c>
@@ -4142,7 +4142,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>189</v>
       </c>
@@ -4153,7 +4153,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>191</v>
       </c>
@@ -4164,7 +4164,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>193</v>
       </c>
@@ -4175,7 +4175,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>195</v>
       </c>
@@ -4186,7 +4186,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>197</v>
       </c>
@@ -4197,7 +4197,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>199</v>
       </c>
@@ -4208,7 +4208,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>201</v>
       </c>
@@ -4219,7 +4219,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>203</v>
       </c>
@@ -4230,7 +4230,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>205</v>
       </c>
@@ -4241,7 +4241,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>207</v>
       </c>
@@ -4252,7 +4252,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>209</v>
       </c>
@@ -4263,7 +4263,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>211</v>
       </c>
@@ -4274,7 +4274,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>213</v>
       </c>
@@ -4285,7 +4285,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>215</v>
       </c>
@@ -4296,7 +4296,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>217</v>
       </c>
@@ -4307,7 +4307,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>219</v>
       </c>
@@ -4318,7 +4318,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>221</v>
       </c>
@@ -4329,7 +4329,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>223</v>
       </c>
@@ -4340,7 +4340,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>225</v>
       </c>
@@ -4351,7 +4351,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>227</v>
       </c>
@@ -4362,7 +4362,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>229</v>
       </c>
@@ -4373,7 +4373,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>231</v>
       </c>
@@ -4384,7 +4384,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>233</v>
       </c>
@@ -4395,7 +4395,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>235</v>
       </c>
@@ -4406,7 +4406,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>237</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>239</v>
       </c>
@@ -4428,7 +4428,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>241</v>
       </c>
@@ -4439,7 +4439,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>243</v>
       </c>
@@ -4450,7 +4450,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>245</v>
       </c>
@@ -4461,7 +4461,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>247</v>
       </c>
@@ -4472,7 +4472,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>249</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>251</v>
       </c>
@@ -4494,7 +4494,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>253</v>
       </c>
@@ -4505,7 +4505,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>255</v>
       </c>
@@ -4516,7 +4516,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>257</v>
       </c>
@@ -4527,7 +4527,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>259</v>
       </c>
@@ -4538,7 +4538,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>261</v>
       </c>
@@ -4549,7 +4549,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>263</v>
       </c>
@@ -4560,7 +4560,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>265</v>
       </c>
@@ -4571,7 +4571,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>267</v>
       </c>
@@ -4582,7 +4582,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>269</v>
       </c>
@@ -4593,7 +4593,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>271</v>
       </c>
@@ -4604,7 +4604,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>273</v>
       </c>
@@ -4615,7 +4615,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>275</v>
       </c>
@@ -4626,7 +4626,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>277</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>279</v>
       </c>
@@ -4648,7 +4648,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>281</v>
       </c>
@@ -4659,7 +4659,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>283</v>
       </c>
@@ -4670,7 +4670,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>285</v>
       </c>
@@ -4681,7 +4681,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>287</v>
       </c>
@@ -4692,7 +4692,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>289</v>
       </c>
@@ -4703,7 +4703,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>291</v>
       </c>
@@ -4714,7 +4714,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>293</v>
       </c>
@@ -4725,7 +4725,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>295</v>
       </c>
@@ -4736,7 +4736,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>297</v>
       </c>
@@ -4747,7 +4747,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>299</v>
       </c>
@@ -4758,7 +4758,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>301</v>
       </c>
@@ -4769,7 +4769,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>303</v>
       </c>
@@ -4780,7 +4780,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>305</v>
       </c>
@@ -4808,7 +4808,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>310</v>
       </c>
@@ -4819,7 +4819,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>312</v>
       </c>
@@ -4830,7 +4830,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>314</v>
       </c>
@@ -4841,7 +4841,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>316</v>
       </c>
@@ -4852,7 +4852,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>318</v>
       </c>
@@ -4863,7 +4863,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>320</v>
       </c>
@@ -4874,7 +4874,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>322</v>
       </c>
@@ -4885,7 +4885,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>324</v>
       </c>
@@ -4896,7 +4896,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>326</v>
       </c>
@@ -4907,7 +4907,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>328</v>
       </c>
@@ -4918,7 +4918,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>330</v>
       </c>
@@ -4929,7 +4929,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>332</v>
       </c>
@@ -4940,7 +4940,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>334</v>
       </c>
@@ -4951,7 +4951,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>336</v>
       </c>
@@ -4962,7 +4962,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>338</v>
       </c>
@@ -4973,7 +4973,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>340</v>
       </c>
@@ -5001,7 +5001,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>345</v>
       </c>
@@ -5012,7 +5012,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>347</v>
       </c>
@@ -5023,7 +5023,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>349</v>
       </c>
@@ -5034,7 +5034,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>351</v>
       </c>
@@ -5045,7 +5045,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>353</v>
       </c>
@@ -5056,7 +5056,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>355</v>
       </c>
@@ -5067,7 +5067,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>357</v>
       </c>
@@ -5078,7 +5078,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>359</v>
       </c>
@@ -5089,7 +5089,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>361</v>
       </c>
@@ -5100,7 +5100,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>363</v>
       </c>
@@ -5111,7 +5111,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>365</v>
       </c>
@@ -5122,7 +5122,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>367</v>
       </c>
@@ -5133,7 +5133,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>369</v>
       </c>
@@ -5144,7 +5144,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>371</v>
       </c>
@@ -5155,7 +5155,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>373</v>
       </c>
@@ -5166,7 +5166,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>375</v>
       </c>
@@ -5177,7 +5177,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>377</v>
       </c>
@@ -5188,7 +5188,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>379</v>
       </c>
@@ -5199,7 +5199,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>381</v>
       </c>
@@ -5210,7 +5210,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>383</v>
       </c>
@@ -5221,7 +5221,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>385</v>
       </c>
@@ -5232,7 +5232,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>387</v>
       </c>
@@ -5243,7 +5243,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>389</v>
       </c>
@@ -5254,7 +5254,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>391</v>
       </c>
@@ -5265,7 +5265,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>393</v>
       </c>
@@ -5276,7 +5276,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>395</v>
       </c>
@@ -5287,7 +5287,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>397</v>
       </c>
@@ -5298,7 +5298,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>399</v>
       </c>
@@ -5309,7 +5309,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>401</v>
       </c>
@@ -5337,7 +5337,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>405</v>
       </c>
@@ -5348,7 +5348,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>407</v>
       </c>
@@ -5359,7 +5359,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>409</v>
       </c>
@@ -5370,7 +5370,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>411</v>
       </c>
@@ -5381,7 +5381,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>413</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>415</v>
       </c>
@@ -5403,7 +5403,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>417</v>
       </c>
@@ -5414,7 +5414,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>419</v>
       </c>
@@ -5425,7 +5425,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>421</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>423</v>
       </c>
@@ -5447,7 +5447,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>425</v>
       </c>
@@ -5458,7 +5458,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>427</v>
       </c>
@@ -5469,7 +5469,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>429</v>
       </c>
@@ -5480,7 +5480,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>431</v>
       </c>
@@ -5491,7 +5491,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>433</v>
       </c>
@@ -5502,7 +5502,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>435</v>
       </c>
@@ -5513,7 +5513,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>437</v>
       </c>
@@ -5524,7 +5524,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>439</v>
       </c>
@@ -5535,7 +5535,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>441</v>
       </c>
@@ -5546,7 +5546,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>443</v>
       </c>
@@ -5557,7 +5557,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>445</v>
       </c>
@@ -5568,7 +5568,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>447</v>
       </c>
@@ -5596,7 +5596,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>452</v>
       </c>
@@ -5607,7 +5607,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>454</v>
       </c>
@@ -5618,7 +5618,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>456</v>
       </c>
@@ -5629,7 +5629,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>458</v>
       </c>
@@ -5640,7 +5640,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>460</v>
       </c>
@@ -5651,7 +5651,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>462</v>
       </c>
@@ -5662,7 +5662,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>464</v>
       </c>
@@ -5673,7 +5673,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>466</v>
       </c>
@@ -5684,7 +5684,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>468</v>
       </c>
@@ -5695,7 +5695,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>470</v>
       </c>
@@ -5706,7 +5706,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>472</v>
       </c>
@@ -5717,7 +5717,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>474</v>
       </c>
@@ -5728,7 +5728,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>476</v>
       </c>
@@ -5739,7 +5739,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>478</v>
       </c>
@@ -5767,7 +5767,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>482</v>
       </c>
@@ -5778,7 +5778,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>484</v>
       </c>
@@ -5789,7 +5789,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>486</v>
       </c>
@@ -5800,7 +5800,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>488</v>
       </c>
@@ -5811,7 +5811,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>490</v>
       </c>
@@ -5822,7 +5822,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>492</v>
       </c>
@@ -5833,7 +5833,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>494</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>496</v>
       </c>
@@ -5855,7 +5855,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>498</v>
       </c>
@@ -5866,7 +5866,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>500</v>
       </c>
@@ -5877,7 +5877,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>502</v>
       </c>
@@ -5888,7 +5888,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>504</v>
       </c>
@@ -5899,7 +5899,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>506</v>
       </c>
@@ -5910,7 +5910,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>508</v>
       </c>
@@ -5921,7 +5921,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>510</v>
       </c>
@@ -5932,7 +5932,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>512</v>
       </c>
@@ -5943,7 +5943,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>514</v>
       </c>
@@ -5954,7 +5954,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>516</v>
       </c>
@@ -5965,7 +5965,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>518</v>
       </c>
@@ -5976,7 +5976,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>520</v>
       </c>
@@ -5987,7 +5987,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>522</v>
       </c>
@@ -5998,7 +5998,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>524</v>
       </c>
@@ -6009,7 +6009,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>526</v>
       </c>
@@ -6020,7 +6020,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>528</v>
       </c>
@@ -6031,7 +6031,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>530</v>
       </c>
@@ -6042,7 +6042,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>532</v>
       </c>
@@ -6070,7 +6070,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>536</v>
       </c>
@@ -6081,7 +6081,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>538</v>
       </c>
@@ -6092,7 +6092,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>540</v>
       </c>
@@ -6103,7 +6103,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>542</v>
       </c>
@@ -6114,7 +6114,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>544</v>
       </c>
@@ -6125,7 +6125,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>546</v>
       </c>
@@ -6136,7 +6136,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>548</v>
       </c>
@@ -6147,7 +6147,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>550</v>
       </c>
@@ -6158,7 +6158,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>552</v>
       </c>
@@ -6169,7 +6169,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>554</v>
       </c>
@@ -6180,7 +6180,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>556</v>
       </c>
@@ -6191,7 +6191,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>558</v>
       </c>
@@ -6202,7 +6202,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>560</v>
       </c>
@@ -6213,7 +6213,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>562</v>
       </c>
@@ -6224,7 +6224,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>564</v>
       </c>
@@ -6235,7 +6235,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>566</v>
       </c>
@@ -6246,7 +6246,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>568</v>
       </c>
@@ -6257,7 +6257,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>570</v>
       </c>
@@ -6268,7 +6268,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>572</v>
       </c>
@@ -6279,7 +6279,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>574</v>
       </c>
@@ -6290,7 +6290,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>576</v>
       </c>
@@ -6301,7 +6301,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>578</v>
       </c>
@@ -6312,7 +6312,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>580</v>
       </c>
@@ -6323,7 +6323,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>582</v>
       </c>
@@ -6334,7 +6334,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>584</v>
       </c>
@@ -6345,7 +6345,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>586</v>
       </c>
@@ -6376,7 +6376,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>592</v>
       </c>
@@ -6387,7 +6387,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>595</v>
       </c>
@@ -6398,7 +6398,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>597</v>
       </c>
@@ -6409,7 +6409,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>599</v>
       </c>
@@ -6437,7 +6437,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>604</v>
       </c>
@@ -6448,7 +6448,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>606</v>
       </c>
@@ -6459,7 +6459,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>608</v>
       </c>
@@ -6470,7 +6470,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>610</v>
       </c>
@@ -6481,7 +6481,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>612</v>
       </c>
@@ -6492,7 +6492,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>614</v>
       </c>
@@ -6503,7 +6503,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>616</v>
       </c>
@@ -6514,7 +6514,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>618</v>
       </c>
@@ -6525,7 +6525,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>620</v>
       </c>
@@ -6536,7 +6536,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>622</v>
       </c>
@@ -6547,7 +6547,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>624</v>
       </c>
@@ -6558,7 +6558,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>626</v>
       </c>
@@ -6569,7 +6569,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>628</v>
       </c>
@@ -6580,7 +6580,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>630</v>
       </c>
@@ -6591,7 +6591,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>632</v>
       </c>
@@ -6602,7 +6602,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>634</v>
       </c>
@@ -6613,7 +6613,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>636</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>638</v>
       </c>
@@ -6635,7 +6635,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>640</v>
       </c>
@@ -6646,7 +6646,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>642</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>644</v>
       </c>
@@ -6668,7 +6668,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>646</v>
       </c>
@@ -6679,7 +6679,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>648</v>
       </c>
@@ -6707,7 +6707,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>653</v>
       </c>
@@ -6718,7 +6718,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>655</v>
       </c>
@@ -6729,7 +6729,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>657</v>
       </c>
@@ -6740,7 +6740,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>659</v>
       </c>
@@ -6751,7 +6751,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>661</v>
       </c>
@@ -6762,7 +6762,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>663</v>
       </c>
@@ -6773,7 +6773,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>665</v>
       </c>
@@ -6784,7 +6784,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>667</v>
       </c>
@@ -6795,7 +6795,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>669</v>
       </c>
@@ -6806,7 +6806,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>671</v>
       </c>
@@ -6817,7 +6817,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>673</v>
       </c>
@@ -6828,7 +6828,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>675</v>
       </c>
@@ -6839,7 +6839,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>677</v>
       </c>
@@ -6850,7 +6850,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>679</v>
       </c>
@@ -6861,7 +6861,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>681</v>
       </c>
@@ -6872,7 +6872,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>683</v>
       </c>
@@ -6883,7 +6883,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>685</v>
       </c>
@@ -6894,7 +6894,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>687</v>
       </c>
@@ -6905,7 +6905,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>689</v>
       </c>
@@ -6916,7 +6916,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>691</v>
       </c>
@@ -6927,7 +6927,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>693</v>
       </c>
@@ -6938,7 +6938,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>695</v>
       </c>
@@ -6949,7 +6949,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>697</v>
       </c>
@@ -6977,7 +6977,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>701</v>
       </c>
@@ -6988,7 +6988,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>703</v>
       </c>
@@ -6999,7 +6999,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>705</v>
       </c>
@@ -7010,7 +7010,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>707</v>
       </c>
@@ -7021,7 +7021,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>709</v>
       </c>
@@ -7032,7 +7032,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>711</v>
       </c>
@@ -7043,7 +7043,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>713</v>
       </c>
@@ -7054,7 +7054,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>715</v>
       </c>
@@ -7065,7 +7065,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>717</v>
       </c>
@@ -7076,7 +7076,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>719</v>
       </c>
@@ -7087,7 +7087,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>721</v>
       </c>
@@ -7098,7 +7098,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>723</v>
       </c>
@@ -7109,7 +7109,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>725</v>
       </c>
@@ -7120,7 +7120,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>727</v>
       </c>
@@ -7131,7 +7131,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="318" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>729</v>
       </c>
@@ -7171,7 +7171,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>736</v>
       </c>
@@ -7182,7 +7182,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>738</v>
       </c>
@@ -7193,7 +7193,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
         <v>740</v>
       </c>
@@ -7224,7 +7224,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="324" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
         <v>745</v>
       </c>
@@ -7235,7 +7235,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="325" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
         <v>747</v>
       </c>
@@ -7246,7 +7246,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="326" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
         <v>749</v>
       </c>
@@ -7257,7 +7257,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="327" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
         <v>751</v>
       </c>
@@ -7268,7 +7268,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="328" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>753</v>
       </c>
@@ -7299,7 +7299,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="330" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
         <v>758</v>
       </c>
@@ -7347,7 +7347,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="333" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
         <v>765</v>
       </c>
@@ -7358,7 +7358,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="334" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
         <v>767</v>
       </c>
@@ -7449,7 +7449,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="339" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A339">
         <v>90936111</v>
       </c>
@@ -7466,7 +7466,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="340" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
         <v>783</v>
       </c>
@@ -7477,7 +7477,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="341" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>785</v>
       </c>
@@ -7492,7 +7492,14 @@
       <c r="A344" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G341" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G341" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Jobs_1, Jobs_2, Jobs_3"/>
+        <filter val="Jobs_2"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -7923,6 +7930,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052CF2D8E3E532648A9A53BA8B542239D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a1fb610553ec5defc474bb1f7a0ddc39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ce6b1c7-1e7d-4e54-8192-c843964c72a7" xmlns:ns3="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d9d4414e518fb510d6d835712213802" ns2:_="" ns3:_="">
     <xsd:import namespace="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
@@ -8151,16 +8167,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEFD0438-3B89-46D3-AFC2-2E1E8BA59BF1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF250B34-2756-44A2-A030-8FEBB211D63C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8177,12 +8192,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEFD0438-3B89-46D3-AFC2-2E1E8BA59BF1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Pulled Jobs_1 data for all peer MSAs. Cleaned data pulling code, and exported final dataframe to excel in long and wide format.
</commit_message>
<xml_diff>
--- a/Indicator_Gen/Python Code/BLS/config/BLS Configuration File.xlsx
+++ b/Indicator_Gen/Python Code/BLS/config/BLS Configuration File.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\Python Code\BLS\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jchoy\Documents\Python Projects\Regional-Monitoring\Indicator_Gen\Python Code\BLS\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF2F604-F4B4-4818-B0F9-5D7F69794DBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34217FC0-D147-4437-A0E5-96D3B87074DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="2400" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="5" r:id="rId1"/>
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="845">
   <si>
     <t>TODO list:</t>
   </si>
@@ -2646,6 +2646,9 @@
   </si>
   <si>
     <t>Notes2</t>
+  </si>
+  <si>
+    <t>Jobs_1, Jobs_2</t>
   </si>
 </sst>
 </file>
@@ -3275,7 +3278,7 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>2014</v>
@@ -3550,7 +3553,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -3629,7 +3632,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>97</v>
       </c>
@@ -3756,7 +3759,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>120</v>
       </c>
@@ -3916,7 +3919,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>149</v>
       </c>
@@ -4791,7 +4794,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>307</v>
       </c>
@@ -4984,7 +4987,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>342</v>
       </c>
@@ -5320,7 +5323,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>403</v>
       </c>
@@ -5579,7 +5582,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>449</v>
       </c>
@@ -5750,7 +5753,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>480</v>
       </c>
@@ -6053,7 +6056,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>534</v>
       </c>
@@ -6356,7 +6359,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>588</v>
       </c>
@@ -6420,7 +6423,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>601</v>
       </c>
@@ -6690,7 +6693,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>650</v>
       </c>
@@ -6960,7 +6963,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>699</v>
       </c>
@@ -7131,7 +7134,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="318" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>729</v>
       </c>
@@ -7151,7 +7154,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>733</v>
       </c>
@@ -7204,7 +7207,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
         <v>742</v>
       </c>
@@ -7279,7 +7282,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="329" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
         <v>755</v>
       </c>
@@ -7310,7 +7313,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="331" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
         <v>760</v>
       </c>
@@ -7327,7 +7330,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="332" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
         <v>762</v>
       </c>
@@ -7369,7 +7372,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="335" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
         <v>769</v>
       </c>
@@ -7389,7 +7392,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="336" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
         <v>772</v>
       </c>
@@ -7409,7 +7412,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="337" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
         <v>775</v>
       </c>
@@ -7429,7 +7432,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="338" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
         <v>778</v>
       </c>
@@ -7496,7 +7499,7 @@
     <filterColumn colId="2">
       <filters>
         <filter val="Jobs_1, Jobs_2, Jobs_3"/>
-        <filter val="Jobs_2"/>
+        <filter val="Jobs_1, Jobs_3"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -7776,7 +7779,7 @@
         <v>819</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>844</v>
       </c>
       <c r="D2" t="s">
         <v>820</v>
@@ -7930,15 +7933,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052CF2D8E3E532648A9A53BA8B542239D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a1fb610553ec5defc474bb1f7a0ddc39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ce6b1c7-1e7d-4e54-8192-c843964c72a7" xmlns:ns3="4ae99fea-3ccc-4497-bfcd-e0cb757e7dff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d9d4414e518fb510d6d835712213802" ns2:_="" ns3:_="">
     <xsd:import namespace="9ce6b1c7-1e7d-4e54-8192-c843964c72a7"/>
@@ -8167,15 +8161,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEFD0438-3B89-46D3-AFC2-2E1E8BA59BF1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF250B34-2756-44A2-A030-8FEBB211D63C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8192,4 +8187,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEFD0438-3B89-46D3-AFC2-2E1E8BA59BF1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Moving some things around, MOE updates to query ACS, minor updates to BLS work
</commit_message>
<xml_diff>
--- a/Indicator_Gen/Python Code/BLS/config/BLS Configuration File.xlsx
+++ b/Indicator_Gen/Python Code/BLS/config/BLS Configuration File.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\Python Code\BLS\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{754DFA71-3D72-4AF0-9546-1E3AE5FED193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47FDC2D5-EC53-480D-B37C-DCBD17E40694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="5" r:id="rId1"/>
@@ -116,7 +116,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="831">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1345" uniqueCount="871">
   <si>
     <t>TODO list:</t>
   </si>
@@ -2609,6 +2609,126 @@
   </si>
   <si>
     <t>confirmed</t>
+  </si>
+  <si>
+    <t>16740</t>
+  </si>
+  <si>
+    <t>Charlotte-Concord-Gastonia, NC-SC Metro Area</t>
+  </si>
+  <si>
+    <t>17140</t>
+  </si>
+  <si>
+    <t>Cincinnati, OH-KY-IN Metro Area</t>
+  </si>
+  <si>
+    <t>17460</t>
+  </si>
+  <si>
+    <t>Cleveland-Elyria, OH Metro Area</t>
+  </si>
+  <si>
+    <t>18140</t>
+  </si>
+  <si>
+    <t>Columbus, OH Metro Area</t>
+  </si>
+  <si>
+    <t>19740</t>
+  </si>
+  <si>
+    <t>Denver-Aurora-Lakewood, CO Metro Area</t>
+  </si>
+  <si>
+    <t>19820</t>
+  </si>
+  <si>
+    <t>Detroit-Warren-Dearborn, MI Metro Area</t>
+  </si>
+  <si>
+    <t>26900</t>
+  </si>
+  <si>
+    <t>Indianapolis-Carmel-Anderson, IN Metro Area</t>
+  </si>
+  <si>
+    <t>28140</t>
+  </si>
+  <si>
+    <t>Kansas City, MO-KS Metro Area</t>
+  </si>
+  <si>
+    <t>33100</t>
+  </si>
+  <si>
+    <t>Miami-Fort Lauderdale-Pompano Beach, FL Metro Area</t>
+  </si>
+  <si>
+    <t>36740</t>
+  </si>
+  <si>
+    <t>Orlando-Kissimmee-Sanford, FL Metro Area</t>
+  </si>
+  <si>
+    <t>38060</t>
+  </si>
+  <si>
+    <t>Phoenix-Mesa-Chandler, AZ Metro Area</t>
+  </si>
+  <si>
+    <t>38300</t>
+  </si>
+  <si>
+    <t>Pittsburgh, PA Metro Area</t>
+  </si>
+  <si>
+    <t>38900</t>
+  </si>
+  <si>
+    <t>Portland-Vancouver-Hillsboro, OR-WA Metro Area</t>
+  </si>
+  <si>
+    <t>40140</t>
+  </si>
+  <si>
+    <t>Riverside-San Bernardino-Ontario, CA Metro Area</t>
+  </si>
+  <si>
+    <t>41180</t>
+  </si>
+  <si>
+    <t>St. Louis, MO-IL Metro Area</t>
+  </si>
+  <si>
+    <t>41620</t>
+  </si>
+  <si>
+    <t>Salt Lake City, UT Metro Area</t>
+  </si>
+  <si>
+    <t>41700</t>
+  </si>
+  <si>
+    <t>San Antonio-New Braunfels, TX Metro Area</t>
+  </si>
+  <si>
+    <t>41740</t>
+  </si>
+  <si>
+    <t>San Diego-Chula Vista-Carlsbad, CA Metro Area</t>
+  </si>
+  <si>
+    <t>41940</t>
+  </si>
+  <si>
+    <t>San Jose-Sunnyvale-Santa Clara, CA Metro Area</t>
+  </si>
+  <si>
+    <t>45300</t>
+  </si>
+  <si>
+    <t>Tampa-St. Petersburg-Clearwater, FL Metro Area</t>
   </si>
 </sst>
 </file>
@@ -3642,10 +3762,10 @@
         <v>801</v>
       </c>
       <c r="G14" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I14">
         <v>2000</v>
@@ -3681,7 +3801,7 @@
         <v>801</v>
       </c>
       <c r="G15" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="H15">
         <v>3</v>
@@ -3954,7 +4074,7 @@
         <v>803</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -3962,7 +4082,7 @@
         <v>804</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -3970,7 +4090,7 @@
         <v>17</v>
       </c>
       <c r="B9">
-        <v>2014</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -4010,7 +4130,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.81640625" bestFit="1" customWidth="1"/>
@@ -4035,25 +4155,185 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>831</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>832</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>833</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>834</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>835</v>
+      </c>
+      <c r="B5" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>837</v>
+      </c>
+      <c r="B6" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>839</v>
+      </c>
+      <c r="B7" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>841</v>
+      </c>
+      <c r="B8" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>843</v>
+      </c>
+      <c r="B9" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>845</v>
+      </c>
+      <c r="B10" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>847</v>
+      </c>
+      <c r="B11" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>849</v>
+      </c>
+      <c r="B12" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>851</v>
+      </c>
+      <c r="B13" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>853</v>
+      </c>
+      <c r="B14" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>855</v>
+      </c>
+      <c r="B15" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>857</v>
+      </c>
+      <c r="B16" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>859</v>
+      </c>
+      <c r="B18" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>861</v>
+      </c>
+      <c r="B19" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>863</v>
+      </c>
+      <c r="B20" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>865</v>
+      </c>
+      <c r="B21" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>867</v>
+      </c>
+      <c r="B23" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>869</v>
+      </c>
+      <c r="B24" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>28</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B25" t="s">
         <v>29</v>
       </c>
     </row>
@@ -4064,7 +4344,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
   <dimension ref="A1:G344"/>
@@ -4136,7 +4416,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -4150,7 +4430,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -4164,7 +4444,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -4195,7 +4475,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>51</v>
       </c>
@@ -4206,7 +4486,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -4217,7 +4497,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>56</v>
       </c>
@@ -4228,7 +4508,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -4239,7 +4519,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>60</v>
       </c>
@@ -4250,7 +4530,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>62</v>
       </c>
@@ -4261,7 +4541,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>64</v>
       </c>
@@ -4272,7 +4552,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>66</v>
       </c>
@@ -4283,7 +4563,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>68</v>
       </c>
@@ -4294,7 +4574,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>70</v>
       </c>
@@ -4322,7 +4602,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>75</v>
       </c>
@@ -4333,7 +4613,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>77</v>
       </c>
@@ -4344,7 +4624,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>79</v>
       </c>
@@ -4355,7 +4635,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>81</v>
       </c>
@@ -4366,7 +4646,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>83</v>
       </c>
@@ -4377,7 +4657,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>85</v>
       </c>
@@ -4388,7 +4668,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>87</v>
       </c>
@@ -4399,7 +4679,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>89</v>
       </c>
@@ -4410,7 +4690,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>91</v>
       </c>
@@ -4421,7 +4701,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>93</v>
       </c>
@@ -4432,7 +4712,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>95</v>
       </c>
@@ -4443,7 +4723,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>97</v>
       </c>
@@ -4454,7 +4734,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>99</v>
       </c>
@@ -4482,7 +4762,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>103</v>
       </c>
@@ -4493,7 +4773,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>105</v>
       </c>
@@ -4504,7 +4784,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>107</v>
       </c>
@@ -4515,7 +4795,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>109</v>
       </c>
@@ -4526,7 +4806,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>111</v>
       </c>
@@ -4537,7 +4817,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>113</v>
       </c>
@@ -4548,7 +4828,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>115</v>
       </c>
@@ -4559,7 +4839,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>117</v>
       </c>
@@ -4570,7 +4850,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>119</v>
       </c>
@@ -4581,7 +4861,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>121</v>
       </c>
@@ -4592,7 +4872,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>123</v>
       </c>
@@ -4603,7 +4883,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>125</v>
       </c>
@@ -4614,7 +4894,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>127</v>
       </c>
@@ -4625,7 +4905,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>129</v>
       </c>
@@ -4636,7 +4916,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>131</v>
       </c>
@@ -4647,7 +4927,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>133</v>
       </c>
@@ -4658,7 +4938,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>135</v>
       </c>
@@ -4669,7 +4949,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>137</v>
       </c>
@@ -4680,7 +4960,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>139</v>
       </c>
@@ -4691,7 +4971,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>141</v>
       </c>
@@ -4702,7 +4982,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>143</v>
       </c>
@@ -4713,7 +4993,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>145</v>
       </c>
@@ -4724,7 +5004,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>147</v>
       </c>
@@ -4735,7 +5015,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>149</v>
       </c>
@@ -4746,7 +5026,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>151</v>
       </c>
@@ -4757,7 +5037,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>153</v>
       </c>
@@ -4768,7 +5048,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>155</v>
       </c>
@@ -4779,7 +5059,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>157</v>
       </c>
@@ -4790,7 +5070,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>159</v>
       </c>
@@ -4801,7 +5081,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>161</v>
       </c>
@@ -4812,7 +5092,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>163</v>
       </c>
@@ -4823,7 +5103,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>165</v>
       </c>
@@ -4834,7 +5114,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>167</v>
       </c>
@@ -4845,7 +5125,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>169</v>
       </c>
@@ -4856,7 +5136,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>171</v>
       </c>
@@ -4867,7 +5147,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>173</v>
       </c>
@@ -4878,7 +5158,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>175</v>
       </c>
@@ -4889,7 +5169,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>177</v>
       </c>
@@ -4900,7 +5180,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>179</v>
       </c>
@@ -4911,7 +5191,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>181</v>
       </c>
@@ -4922,7 +5202,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>183</v>
       </c>
@@ -4933,7 +5213,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>185</v>
       </c>
@@ -4944,7 +5224,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>187</v>
       </c>
@@ -4955,7 +5235,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>189</v>
       </c>
@@ -4966,7 +5246,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>191</v>
       </c>
@@ -4977,7 +5257,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>193</v>
       </c>
@@ -4988,7 +5268,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>195</v>
       </c>
@@ -4999,7 +5279,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>197</v>
       </c>
@@ -5010,7 +5290,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>199</v>
       </c>
@@ -5021,7 +5301,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>201</v>
       </c>
@@ -5032,7 +5312,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>203</v>
       </c>
@@ -5043,7 +5323,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>205</v>
       </c>
@@ -5054,7 +5334,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>207</v>
       </c>
@@ -5065,7 +5345,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>209</v>
       </c>
@@ -5076,7 +5356,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>211</v>
       </c>
@@ -5087,7 +5367,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>213</v>
       </c>
@@ -5098,7 +5378,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>215</v>
       </c>
@@ -5109,7 +5389,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>217</v>
       </c>
@@ -5120,7 +5400,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>219</v>
       </c>
@@ -5131,7 +5411,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>221</v>
       </c>
@@ -5142,7 +5422,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>223</v>
       </c>
@@ -5153,7 +5433,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>225</v>
       </c>
@@ -5164,7 +5444,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>227</v>
       </c>
@@ -5175,7 +5455,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>229</v>
       </c>
@@ -5186,7 +5466,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>231</v>
       </c>
@@ -5197,7 +5477,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>233</v>
       </c>
@@ -5208,7 +5488,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>235</v>
       </c>
@@ -5219,7 +5499,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>237</v>
       </c>
@@ -5230,7 +5510,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>239</v>
       </c>
@@ -5241,7 +5521,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>241</v>
       </c>
@@ -5252,7 +5532,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>243</v>
       </c>
@@ -5263,7 +5543,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>245</v>
       </c>
@@ -5274,7 +5554,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>247</v>
       </c>
@@ -5285,7 +5565,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>249</v>
       </c>
@@ -5296,7 +5576,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>251</v>
       </c>
@@ -5307,7 +5587,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>253</v>
       </c>
@@ -5318,7 +5598,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>255</v>
       </c>
@@ -5329,7 +5609,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>257</v>
       </c>
@@ -5357,7 +5637,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>262</v>
       </c>
@@ -5368,7 +5648,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>264</v>
       </c>
@@ -5379,7 +5659,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>266</v>
       </c>
@@ -5390,7 +5670,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>268</v>
       </c>
@@ -5401,7 +5681,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>270</v>
       </c>
@@ -5412,7 +5692,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>272</v>
       </c>
@@ -5423,7 +5703,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>274</v>
       </c>
@@ -5434,7 +5714,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>276</v>
       </c>
@@ -5445,7 +5725,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>278</v>
       </c>
@@ -5456,7 +5736,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>280</v>
       </c>
@@ -5467,7 +5747,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>282</v>
       </c>
@@ -5478,7 +5758,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>284</v>
       </c>
@@ -5489,7 +5769,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>286</v>
       </c>
@@ -5500,7 +5780,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>288</v>
       </c>
@@ -5511,7 +5791,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>290</v>
       </c>
@@ -5522,7 +5802,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>292</v>
       </c>
@@ -5550,7 +5830,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>297</v>
       </c>
@@ -5561,7 +5841,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>299</v>
       </c>
@@ -5572,7 +5852,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>301</v>
       </c>
@@ -5583,7 +5863,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>303</v>
       </c>
@@ -5594,7 +5874,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>305</v>
       </c>
@@ -5605,7 +5885,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>307</v>
       </c>
@@ -5616,7 +5896,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="135" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>309</v>
       </c>
@@ -5627,7 +5907,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="136" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>311</v>
       </c>
@@ -5638,7 +5918,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>313</v>
       </c>
@@ -5649,7 +5929,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>315</v>
       </c>
@@ -5660,7 +5940,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>317</v>
       </c>
@@ -5671,7 +5951,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>319</v>
       </c>
@@ -5682,7 +5962,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>321</v>
       </c>
@@ -5693,7 +5973,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>323</v>
       </c>
@@ -5704,7 +5984,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="143" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>325</v>
       </c>
@@ -5715,7 +5995,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>327</v>
       </c>
@@ -5726,7 +6006,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="145" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>329</v>
       </c>
@@ -5737,7 +6017,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>331</v>
       </c>
@@ -5748,7 +6028,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="147" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>333</v>
       </c>
@@ -5759,7 +6039,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="148" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>335</v>
       </c>
@@ -5770,7 +6050,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="149" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>337</v>
       </c>
@@ -5781,7 +6061,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="150" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>339</v>
       </c>
@@ -5792,7 +6072,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="151" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>341</v>
       </c>
@@ -5803,7 +6083,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="152" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>343</v>
       </c>
@@ -5814,7 +6094,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="153" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>345</v>
       </c>
@@ -5825,7 +6105,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="154" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>347</v>
       </c>
@@ -5836,7 +6116,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="155" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>349</v>
       </c>
@@ -5847,7 +6127,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="156" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>351</v>
       </c>
@@ -5858,7 +6138,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="157" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>353</v>
       </c>
@@ -5886,7 +6166,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="159" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>357</v>
       </c>
@@ -5897,7 +6177,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="160" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>359</v>
       </c>
@@ -5908,7 +6188,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="161" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>361</v>
       </c>
@@ -5919,7 +6199,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="162" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>363</v>
       </c>
@@ -5930,7 +6210,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="163" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>365</v>
       </c>
@@ -5941,7 +6221,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="164" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>367</v>
       </c>
@@ -5952,7 +6232,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="165" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>369</v>
       </c>
@@ -5963,7 +6243,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="166" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>371</v>
       </c>
@@ -5974,7 +6254,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="167" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>373</v>
       </c>
@@ -5985,7 +6265,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="168" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>375</v>
       </c>
@@ -5996,7 +6276,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="169" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>377</v>
       </c>
@@ -6007,7 +6287,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="170" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>379</v>
       </c>
@@ -6018,7 +6298,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="171" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>381</v>
       </c>
@@ -6029,7 +6309,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="172" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>383</v>
       </c>
@@ -6040,7 +6320,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="173" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>385</v>
       </c>
@@ -6051,7 +6331,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="174" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>387</v>
       </c>
@@ -6062,7 +6342,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="175" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>389</v>
       </c>
@@ -6073,7 +6353,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="176" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>391</v>
       </c>
@@ -6084,7 +6364,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="177" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>393</v>
       </c>
@@ -6095,7 +6375,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="178" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>395</v>
       </c>
@@ -6106,7 +6386,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="179" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>397</v>
       </c>
@@ -6117,7 +6397,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="180" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>399</v>
       </c>
@@ -6145,7 +6425,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="182" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>404</v>
       </c>
@@ -6156,7 +6436,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>406</v>
       </c>
@@ -6167,7 +6447,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="184" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>408</v>
       </c>
@@ -6178,7 +6458,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>410</v>
       </c>
@@ -6189,7 +6469,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>412</v>
       </c>
@@ -6200,7 +6480,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>414</v>
       </c>
@@ -6211,7 +6491,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="188" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>416</v>
       </c>
@@ -6222,7 +6502,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="189" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>418</v>
       </c>
@@ -6233,7 +6513,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="190" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>420</v>
       </c>
@@ -6244,7 +6524,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="191" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>422</v>
       </c>
@@ -6255,7 +6535,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="192" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>424</v>
       </c>
@@ -6266,7 +6546,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>426</v>
       </c>
@@ -6277,7 +6557,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>428</v>
       </c>
@@ -6288,7 +6568,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>430</v>
       </c>
@@ -6316,7 +6596,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>434</v>
       </c>
@@ -6327,7 +6607,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="198" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>436</v>
       </c>
@@ -6338,7 +6618,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>438</v>
       </c>
@@ -6349,7 +6629,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="200" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>440</v>
       </c>
@@ -6360,7 +6640,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="201" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>442</v>
       </c>
@@ -6371,7 +6651,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="202" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>444</v>
       </c>
@@ -6382,7 +6662,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="203" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>446</v>
       </c>
@@ -6393,7 +6673,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="204" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>448</v>
       </c>
@@ -6404,7 +6684,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="205" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>450</v>
       </c>
@@ -6415,7 +6695,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="206" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>452</v>
       </c>
@@ -6426,7 +6706,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="207" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>454</v>
       </c>
@@ -6437,7 +6717,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="208" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>456</v>
       </c>
@@ -6448,7 +6728,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="209" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>458</v>
       </c>
@@ -6459,7 +6739,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="210" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>460</v>
       </c>
@@ -6470,7 +6750,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="211" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>462</v>
       </c>
@@ -6481,7 +6761,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>464</v>
       </c>
@@ -6492,7 +6772,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>466</v>
       </c>
@@ -6503,7 +6783,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="214" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>468</v>
       </c>
@@ -6514,7 +6794,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="215" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>470</v>
       </c>
@@ -6525,7 +6805,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="216" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>472</v>
       </c>
@@ -6536,7 +6816,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="217" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>474</v>
       </c>
@@ -6547,7 +6827,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="218" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>476</v>
       </c>
@@ -6558,7 +6838,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="219" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>478</v>
       </c>
@@ -6569,7 +6849,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="220" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>480</v>
       </c>
@@ -6580,7 +6860,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="221" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>482</v>
       </c>
@@ -6591,7 +6871,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="222" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>484</v>
       </c>
@@ -6619,7 +6899,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="224" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>488</v>
       </c>
@@ -6630,7 +6910,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="225" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>490</v>
       </c>
@@ -6641,7 +6921,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="226" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>492</v>
       </c>
@@ -6652,7 +6932,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="227" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>494</v>
       </c>
@@ -6663,7 +6943,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="228" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>496</v>
       </c>
@@ -6674,7 +6954,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="229" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>498</v>
       </c>
@@ -6685,7 +6965,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="230" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>500</v>
       </c>
@@ -6696,7 +6976,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="231" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>502</v>
       </c>
@@ -6707,7 +6987,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>504</v>
       </c>
@@ -6718,7 +6998,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>506</v>
       </c>
@@ -6729,7 +7009,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>508</v>
       </c>
@@ -6740,7 +7020,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>510</v>
       </c>
@@ -6751,7 +7031,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="236" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>512</v>
       </c>
@@ -6762,7 +7042,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="237" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>514</v>
       </c>
@@ -6773,7 +7053,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="238" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>516</v>
       </c>
@@ -6784,7 +7064,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="239" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>518</v>
       </c>
@@ -6795,7 +7075,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="240" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>520</v>
       </c>
@@ -6806,7 +7086,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="241" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>522</v>
       </c>
@@ -6817,7 +7097,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="242" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>524</v>
       </c>
@@ -6828,7 +7108,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="243" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>526</v>
       </c>
@@ -6839,7 +7119,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="244" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>528</v>
       </c>
@@ -6850,7 +7130,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="245" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>530</v>
       </c>
@@ -6861,7 +7141,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="246" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>532</v>
       </c>
@@ -6872,7 +7152,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="247" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>534</v>
       </c>
@@ -6883,7 +7163,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="248" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>536</v>
       </c>
@@ -6894,7 +7174,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="249" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>538</v>
       </c>
@@ -6925,7 +7205,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="251" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>544</v>
       </c>
@@ -6936,7 +7216,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="252" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>547</v>
       </c>
@@ -6947,7 +7227,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="253" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>549</v>
       </c>
@@ -6958,7 +7238,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="254" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>551</v>
       </c>
@@ -6986,7 +7266,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="256" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>556</v>
       </c>
@@ -6997,7 +7277,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="257" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>558</v>
       </c>
@@ -7008,7 +7288,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="258" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>560</v>
       </c>
@@ -7019,7 +7299,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="259" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>562</v>
       </c>
@@ -7030,7 +7310,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="260" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>564</v>
       </c>
@@ -7041,7 +7321,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="261" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>566</v>
       </c>
@@ -7052,7 +7332,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="262" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>568</v>
       </c>
@@ -7063,7 +7343,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="263" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>570</v>
       </c>
@@ -7074,7 +7354,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="264" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>572</v>
       </c>
@@ -7085,7 +7365,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="265" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>574</v>
       </c>
@@ -7096,7 +7376,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="266" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>576</v>
       </c>
@@ -7107,7 +7387,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="267" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>578</v>
       </c>
@@ -7118,7 +7398,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="268" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>580</v>
       </c>
@@ -7129,7 +7409,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="269" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>582</v>
       </c>
@@ -7140,7 +7420,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="270" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>584</v>
       </c>
@@ -7151,7 +7431,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="271" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>586</v>
       </c>
@@ -7162,7 +7442,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="272" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>588</v>
       </c>
@@ -7173,7 +7453,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="273" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>590</v>
       </c>
@@ -7184,7 +7464,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="274" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>592</v>
       </c>
@@ -7195,7 +7475,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="275" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>594</v>
       </c>
@@ -7206,7 +7486,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="276" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>596</v>
       </c>
@@ -7217,7 +7497,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="277" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>598</v>
       </c>
@@ -7228,7 +7508,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="278" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>600</v>
       </c>
@@ -7256,7 +7536,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="280" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>605</v>
       </c>
@@ -7267,7 +7547,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="281" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>607</v>
       </c>
@@ -7278,7 +7558,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="282" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>609</v>
       </c>
@@ -7289,7 +7569,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="283" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>611</v>
       </c>
@@ -7300,7 +7580,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="284" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>613</v>
       </c>
@@ -7311,7 +7591,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="285" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>615</v>
       </c>
@@ -7322,7 +7602,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="286" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>617</v>
       </c>
@@ -7333,7 +7613,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="287" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>619</v>
       </c>
@@ -7344,7 +7624,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="288" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>621</v>
       </c>
@@ -7355,7 +7635,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="289" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>623</v>
       </c>
@@ -7366,7 +7646,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="290" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>625</v>
       </c>
@@ -7377,7 +7657,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="291" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>627</v>
       </c>
@@ -7388,7 +7668,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="292" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>629</v>
       </c>
@@ -7399,7 +7679,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="293" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>631</v>
       </c>
@@ -7410,7 +7690,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="294" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>633</v>
       </c>
@@ -7421,7 +7701,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="295" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>635</v>
       </c>
@@ -7432,7 +7712,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="296" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>637</v>
       </c>
@@ -7443,7 +7723,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="297" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>639</v>
       </c>
@@ -7454,7 +7734,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="298" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>641</v>
       </c>
@@ -7465,7 +7745,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="299" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>643</v>
       </c>
@@ -7476,7 +7756,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="300" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>645</v>
       </c>
@@ -7487,7 +7767,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="301" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>647</v>
       </c>
@@ -7498,7 +7778,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="302" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>649</v>
       </c>
@@ -7526,7 +7806,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="304" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>653</v>
       </c>
@@ -7537,7 +7817,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="305" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>655</v>
       </c>
@@ -7548,7 +7828,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="306" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>657</v>
       </c>
@@ -7559,7 +7839,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="307" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>659</v>
       </c>
@@ -7570,7 +7850,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="308" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>661</v>
       </c>
@@ -7581,7 +7861,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="309" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>663</v>
       </c>
@@ -7592,7 +7872,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="310" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>665</v>
       </c>
@@ -7603,7 +7883,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="311" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>667</v>
       </c>
@@ -7614,7 +7894,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="312" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>669</v>
       </c>
@@ -7625,7 +7905,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="313" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>671</v>
       </c>
@@ -7636,7 +7916,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="314" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>673</v>
       </c>
@@ -7647,7 +7927,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="315" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>675</v>
       </c>
@@ -7658,7 +7938,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="316" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>677</v>
       </c>
@@ -7669,7 +7949,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="317" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>679</v>
       </c>
@@ -7680,7 +7960,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="318" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>681</v>
       </c>
@@ -7720,7 +8000,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="320" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>688</v>
       </c>
@@ -7731,7 +8011,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="321" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>690</v>
       </c>
@@ -7742,7 +8022,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="322" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
         <v>692</v>
       </c>
@@ -7773,7 +8053,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="324" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
         <v>697</v>
       </c>
@@ -7784,7 +8064,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="325" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
         <v>699</v>
       </c>
@@ -7795,7 +8075,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="326" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
         <v>701</v>
       </c>
@@ -7806,7 +8086,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="327" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
         <v>703</v>
       </c>
@@ -7817,7 +8097,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="328" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>705</v>
       </c>
@@ -7848,7 +8128,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="330" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
         <v>710</v>
       </c>
@@ -7896,7 +8176,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="333" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
         <v>717</v>
       </c>
@@ -7907,7 +8187,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="334" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
         <v>719</v>
       </c>
@@ -7998,7 +8278,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="339" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A339">
         <v>90936111</v>
       </c>
@@ -8015,7 +8295,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="340" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
         <v>734</v>
       </c>
@@ -8026,7 +8306,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="341" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>736</v>
       </c>
@@ -8041,14 +8321,7 @@
       <c r="A344" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G341" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Jobs_1, Jobs_2, Jobs_3"/>
-        <filter val="Jobs_2"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G341" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>